<commit_message>
update fluid interactions, improve collision logic
</commit_message>
<xml_diff>
--- a/raw/Fluid_Interactions.xlsx
+++ b/raw/Fluid_Interactions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\FabricModding\Spectrum\raw\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\FabricModding\Spectrum\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81D34BEC-D649-4B19-99FD-4CEBE1FCB1DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14A9EAF0-5F22-4A31-83A6-628439D9A23B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="34395" windowHeight="21000" xr2:uid="{C062C883-C536-49F0-A3FB-1F783D9E299D}"/>
+    <workbookView xWindow="51480" yWindow="5100" windowWidth="29040" windowHeight="15840" xr2:uid="{C062C883-C536-49F0-A3FB-1F783D9E299D}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="27">
   <si>
     <t>Water</t>
   </si>
@@ -51,12 +51,6 @@
     <t>Cobblestone</t>
   </si>
   <si>
-    <t>Dirt</t>
-  </si>
-  <si>
-    <t>Coarse Dirt</t>
-  </si>
-  <si>
     <t>Frostbite Crystal / Calcite</t>
   </si>
   <si>
@@ -84,9 +78,6 @@
     <t>Blazing Crystal / Cobbled Deepslate</t>
   </si>
   <si>
-    <t>Soul Sand</t>
-  </si>
-  <si>
     <t>Granite</t>
   </si>
   <si>
@@ -105,7 +96,16 @@
     <t>Slush</t>
   </si>
   <si>
-    <t>Dragonrot Dipping:</t>
+    <t>Dirt / Coarse Dirt</t>
+  </si>
+  <si>
+    <t>Sludge</t>
+  </si>
+  <si>
+    <t>Blackslag / Cobbled Blackslag</t>
+  </si>
+  <si>
+    <t>Blackslag</t>
   </si>
 </sst>
 </file>
@@ -147,9 +147,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -183,7 +184,7 @@
     <tableColumn id="1" xr3:uid="{DE5336A1-6B69-497A-A5C3-74A7FE410F18}" name="Fluid Interaction"/>
     <tableColumn id="2" xr3:uid="{26F5AF11-BA60-47DB-8D1A-8BB58E320738}" name="Water" dataDxfId="0"/>
     <tableColumn id="3" xr3:uid="{33C24CD7-EDFD-4792-9ADC-C87D5D38D408}" name="Lava"/>
-    <tableColumn id="4" xr3:uid="{F04C1BC9-7134-4B5E-8F1F-10BF9B37D363}" name="Mud"/>
+    <tableColumn id="4" xr3:uid="{F04C1BC9-7134-4B5E-8F1F-10BF9B37D363}" name="Sludge"/>
     <tableColumn id="5" xr3:uid="{CE658F72-DE59-48BA-9F7E-6C49224C60DA}" name="Liquid Crystal"/>
     <tableColumn id="6" xr3:uid="{FCD23A48-04C8-4A3A-85D5-312C123BC939}" name="Midnight Solution"/>
     <tableColumn id="7" xr3:uid="{B77C0BB1-CAD3-41BF-A72A-FDF51659F30C}" name="Dragonrot"/>
@@ -489,13 +490,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{398016E1-6FAD-49C3-B1B5-A6EC3CDF6D98}">
-  <dimension ref="B2:H25"/>
+  <dimension ref="B2:H15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="32.85546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="19.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.85546875" bestFit="1" customWidth="1"/>
@@ -512,7 +513,7 @@
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="F2" t="s">
         <v>3</v>
@@ -533,16 +534,16 @@
         <v>7</v>
       </c>
       <c r="E3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" t="s">
         <v>8</v>
       </c>
-      <c r="F3" t="s">
-        <v>10</v>
-      </c>
       <c r="G3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H3" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="2:8" x14ac:dyDescent="0.25">
@@ -552,33 +553,33 @@
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="F4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="G4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H4" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
       <c r="F5" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="G5" t="s">
-        <v>17</v>
-      </c>
-      <c r="H5" t="s">
-        <v>2</v>
+        <v>18</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.25">
@@ -590,10 +591,10 @@
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
       <c r="G6" t="s">
-        <v>13</v>
-      </c>
-      <c r="H6" t="s">
-        <v>22</v>
+        <v>11</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.25">
@@ -606,7 +607,7 @@
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
       <c r="H7" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
@@ -622,53 +623,39 @@
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B22" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
         <v>26</v>
-      </c>
-    </row>
-    <row r="23" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B23" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="24" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B24" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="25" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B25" t="s">
-        <v>2</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Liquid Crystal + Water => Clay Liquid Crystal + Lava => Calcite
</commit_message>
<xml_diff>
--- a/raw/Fluid_Interactions.xlsx
+++ b/raw/Fluid_Interactions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\FabricModding\Spectrum\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14A9EAF0-5F22-4A31-83A6-628439D9A23B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AB28FF7-C3C9-4EB4-98BE-4496C294EAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51480" yWindow="5100" windowWidth="29040" windowHeight="15840" xr2:uid="{C062C883-C536-49F0-A3FB-1F783D9E299D}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{C062C883-C536-49F0-A3FB-1F783D9E299D}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="26">
   <si>
     <t>Water</t>
   </si>
@@ -51,12 +51,6 @@
     <t>Cobblestone</t>
   </si>
   <si>
-    <t>Frostbite Crystal / Calcite</t>
-  </si>
-  <si>
-    <t>Clay</t>
-  </si>
-  <si>
     <t>Terracotta</t>
   </si>
   <si>
@@ -75,9 +69,6 @@
     <t>Black Materia</t>
   </si>
   <si>
-    <t>Blazing Crystal / Cobbled Deepslate</t>
-  </si>
-  <si>
     <t>Granite</t>
   </si>
   <si>
@@ -90,22 +81,28 @@
     <t>Tuff</t>
   </si>
   <si>
-    <t>Do not yet exist:</t>
-  </si>
-  <si>
     <t>Slush</t>
   </si>
   <si>
     <t>Dirt / Coarse Dirt</t>
   </si>
   <si>
-    <t>Sludge</t>
-  </si>
-  <si>
     <t>Blackslag / Cobbled Blackslag</t>
   </si>
   <si>
     <t>Blackslag</t>
+  </si>
+  <si>
+    <t>Good Candidates:</t>
+  </si>
+  <si>
+    <t>Frostbite Crystal / Clay</t>
+  </si>
+  <si>
+    <t>Blazing Crystal / Calcite</t>
+  </si>
+  <si>
+    <t>Deepslate / Cobbled Deepslate</t>
   </si>
 </sst>
 </file>
@@ -147,10 +144,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -178,13 +174,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8636DC8E-F786-4DAE-82AB-68EB92F50B00}" name="Tabelle1" displayName="Tabelle1" ref="B2:H8" totalsRowShown="0">
-  <autoFilter ref="B2:H8" xr:uid="{8636DC8E-F786-4DAE-82AB-68EB92F50B00}"/>
-  <tableColumns count="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8636DC8E-F786-4DAE-82AB-68EB92F50B00}" name="Tabelle1" displayName="Tabelle1" ref="B2:G7" totalsRowShown="0">
+  <autoFilter ref="B2:G7" xr:uid="{8636DC8E-F786-4DAE-82AB-68EB92F50B00}"/>
+  <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{DE5336A1-6B69-497A-A5C3-74A7FE410F18}" name="Fluid Interaction"/>
     <tableColumn id="2" xr3:uid="{26F5AF11-BA60-47DB-8D1A-8BB58E320738}" name="Water" dataDxfId="0"/>
     <tableColumn id="3" xr3:uid="{33C24CD7-EDFD-4792-9ADC-C87D5D38D408}" name="Lava"/>
-    <tableColumn id="4" xr3:uid="{F04C1BC9-7134-4B5E-8F1F-10BF9B37D363}" name="Sludge"/>
     <tableColumn id="5" xr3:uid="{CE658F72-DE59-48BA-9F7E-6C49224C60DA}" name="Liquid Crystal"/>
     <tableColumn id="6" xr3:uid="{FCD23A48-04C8-4A3A-85D5-312C123BC939}" name="Midnight Solution"/>
     <tableColumn id="7" xr3:uid="{B77C0BB1-CAD3-41BF-A72A-FDF51659F30C}" name="Dragonrot"/>
@@ -490,19 +485,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{398016E1-6FAD-49C3-B1B5-A6EC3CDF6D98}">
-  <dimension ref="B2:H15"/>
+  <dimension ref="B2:G19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="32.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="32.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>6</v>
       </c>
@@ -513,19 +507,16 @@
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="F2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>0</v>
       </c>
@@ -537,37 +528,31 @@
         <v>23</v>
       </c>
       <c r="F3" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="G3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.25">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>1</v>
       </c>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" t="s">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="F4" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="G4" t="s">
-        <v>13</v>
-      </c>
-      <c r="H4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
@@ -576,79 +561,84 @@
         <v>9</v>
       </c>
       <c r="G5" t="s">
-        <v>18</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
       <c r="G6" t="s">
-        <v>11</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
-      <c r="H7" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B8" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
-    </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="16" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B15" t="s">
-        <v>26</v>
+    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>